<commit_message>
Add 10 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 68
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-alc.report.xlsx
+++ b/tools/importer/reports/import-alc.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="63">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,15 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>error</t>
+  </si>
+  <si>
+    <t>errorStack</t>
+  </si>
+  <si>
+    <t>fragments</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -43,6 +52,9 @@
     <t>["carousel-hero","carousel-winners","cards-game","cards-promo"]</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>index</t>
   </si>
   <si>
@@ -52,13 +64,148 @@
     <t>alc</t>
   </si>
   <si>
-    <t>2026-09-24T21:43:04.733Z</t>
+    <t>2026-09-25T14:58:22.775Z</t>
   </si>
   <si>
     <t>Atlantic Lottery | Buy Tickets Online, Winning Numbers &amp; More</t>
   </si>
   <si>
     <t>https://www.alc.ca/content/alc/en.html</t>
+  </si>
+  <si>
+    <t>our-games/lotto/lotto-6-49.report.json</t>
+  </si>
+  <si>
+    <t>["widget","widget","tabs-game","columns-winner","cards-game"]</t>
+  </si>
+  <si>
+    <t>["prize-payout","winners","how-to-play","odds-of-winning","combination-play"]</t>
+  </si>
+  <si>
+    <t>our-games/lotto/lotto-6-49</t>
+  </si>
+  <si>
+    <t>lotto</t>
+  </si>
+  <si>
+    <t>2026-09-25T14:55:03.790Z</t>
+  </si>
+  <si>
+    <t>Lotto 649 | Our Games | Atlantic Lottery Corporation</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/our-games/lotto/lotto-6-49.html</t>
+  </si>
+  <si>
+    <t>fragments/lotto/lotto-6-49/combination-play.report.json</t>
+  </si>
+  <si>
+    <t>["table-prize"]</t>
+  </si>
+  <si>
+    <t>fragments/lotto/lotto-6-49/combination-play</t>
+  </si>
+  <si>
+    <t>lotto-fragment</t>
+  </si>
+  <si>
+    <t>2026-09-25T14:58:13.277Z</t>
+  </si>
+  <si>
+    <t>lotto-6-49 combination-play</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/our-games/lotto/lotto-6-49.html?fragment=combination-play</t>
+  </si>
+  <si>
+    <t>fragments/lotto/lotto-6-49/how-to-play.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-game","embed-video"]</t>
+  </si>
+  <si>
+    <t>fragments/lotto/lotto-6-49/how-to-play</t>
+  </si>
+  <si>
+    <t>2026-09-25T14:57:06.874Z</t>
+  </si>
+  <si>
+    <t>lotto-6-49 how-to-play</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/our-games/lotto/lotto-6-49.html?fragment=how-to-play</t>
+  </si>
+  <si>
+    <t>fragments/lotto/lotto-6-49/odds-of-winning.report.json</t>
+  </si>
+  <si>
+    <t>fragments/lotto/lotto-6-49/odds-of-winning</t>
+  </si>
+  <si>
+    <t>2026-09-25T14:58:01.878Z</t>
+  </si>
+  <si>
+    <t>lotto-6-49 odds-of-winning</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/our-games/lotto/lotto-6-49.html?fragment=odds-of-winning</t>
+  </si>
+  <si>
+    <t>fragments/lotto/lotto-6-49/prize-payout.report.json</t>
+  </si>
+  <si>
+    <t>["widget"]</t>
+  </si>
+  <si>
+    <t>fragments/lotto/lotto-6-49/prize-payout</t>
+  </si>
+  <si>
+    <t>2026-09-25T14:55:15.077Z</t>
+  </si>
+  <si>
+    <t>lotto-6-49 prize-payout</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/our-games/lotto/lotto-6-49.html?fragment=prize-payout</t>
+  </si>
+  <si>
+    <t>fragments/lotto/lotto-6-49/winners.report.json</t>
+  </si>
+  <si>
+    <t>fragments/lotto/lotto-6-49/winners</t>
+  </si>
+  <si>
+    <t>2026-09-25T14:56:12.083Z</t>
+  </si>
+  <si>
+    <t>lotto-6-49 winners</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/our-games/lotto/lotto-6-49.html?fragment=winners</t>
+  </si>
+  <si>
+    <t>content/alc/en/our-games/lotto/lotto-6-49.html.report.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: Cannot read properties of undefined (reading 'replace')
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: Cannot read properties of undefined (reading 'replace')
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30
+    at processUrl (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:693:31)
+    at async main (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:956:22)</t>
+  </si>
+  <si>
+    <t>content/alc/en/our-games/lotto/lotto-6-49.html</t>
+  </si>
+  <si>
+    <t>failed</t>
+  </si>
+  <si>
+    <t>2026-09-25T14:47:18.414Z</t>
   </si>
 </sst>
 </file>
@@ -447,19 +594,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="1" max="5" width="50" customWidth="1"/>
+    <col min="6" max="6" width="48" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="11" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -484,35 +629,298 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" t="s">
         <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" t="s">
+        <v>44</v>
+      </c>
+      <c r="K6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>31</v>
+      </c>
+      <c r="I8" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" t="s">
+        <v>55</v>
+      </c>
+      <c r="K8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" t="s">
+        <v>62</v>
+      </c>
+      <c r="J9" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>